<commit_message>
Actualizacion automatica de Precios Objetivo (2026-09-01)
</commit_message>
<xml_diff>
--- a/data/precios_objetivo.xlsx
+++ b/data/precios_objetivo.xlsx
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>133.5</v>
+        <v>125.5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2385</v>
+        <v>2380</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>346.3613</v>
+        <v>333.48</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2930</v>
+        <v>2850</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>41.12</v>
+        <v>41.21</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>307</v>
+        <v>326</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -724,7 +724,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>strong_buy</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>10.94</v>
+        <v>11.345</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>13.42143</v>
+        <v>13.13571</v>
       </c>
       <c r="G8" t="n">
         <v>10.5</v>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>267.75</v>
+        <v>261.5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>22.25</v>
+        <v>21.85</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>37.63</v>
+        <v>37.4051</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3.8524</v>
+        <v>4</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -944,7 +944,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3355</v>
+        <v>3725</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>62</v>
+        <v>64.8</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>43.5</v>
+        <v>44.2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1067,10 +1067,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>67.8008</v>
+        <v>67.9742</v>
       </c>
       <c r="G15" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H15" t="n">
         <v>103</v>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>580.5</v>
+        <v>564</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>213.88</v>
+        <v>198.67</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>237.80556</v>
+        <v>238.5</v>
       </c>
       <c r="G17" t="n">
         <v>188</v>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>23.33</v>
+        <v>23.41</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.4099</v>
+        <v>0.4201</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>872.5</v>
+        <v>840</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>696</v>
+        <v>674</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>90.425</v>
+        <v>87.78</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>4.25</v>
+        <v>4.16</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>127.02</v>
+        <v>144.8</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3410</v>
+        <v>3285</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>212.34</v>
+        <v>217.12</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1635,16 +1635,16 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>304.72882</v>
+        <v>323.41898</v>
       </c>
       <c r="G28" t="n">
         <v>180</v>
       </c>
       <c r="H28" t="n">
-        <v>500</v>
+        <v>515</v>
       </c>
       <c r="I28" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>799</v>
+        <v>860</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>260.55</v>
+        <v>253.89</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>327.004</v>
+        <v>327.6707</v>
       </c>
       <c r="G30" t="n">
         <v>230</v>
@@ -1763,7 +1763,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>13.325</v>
+        <v>13.785</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1766</v>
+        <v>1841</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>154.21</v>
+        <v>141.6</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>7.8</v>
+        <v>7.92</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>9.574999999999999</v>
+        <v>10.205</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1165</v>
+        <v>1255</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>768.8049999999999</v>
+        <v>765.725</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2071,7 +2071,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>3050</v>
+        <v>2970</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>8.619999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2119,10 +2119,10 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>12.905</v>
+        <v>12.3598</v>
       </c>
       <c r="G39" t="n">
-        <v>10.6</v>
+        <v>10</v>
       </c>
       <c r="H39" t="n">
         <v>15</v>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1700</v>
+        <v>1792</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>4.455</v>
+        <v>4.1201</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2233,13 +2233,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>7.3820453</v>
+        <v>7.3793902</v>
       </c>
       <c r="G42" t="n">
-        <v>4.056258</v>
+        <v>4.0552907</v>
       </c>
       <c r="H42" t="n">
-        <v>10.097938</v>
+        <v>10.095529</v>
       </c>
       <c r="I42" t="n">
         <v>24</v>
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2234</v>
+        <v>2336</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1780</v>
+        <v>1815</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>312.16</v>
+        <v>290.675</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>371.35483</v>
+        <v>371.19354</v>
       </c>
       <c r="G45" t="n">
         <v>290</v>
@@ -2401,7 +2401,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4257.5</v>
+        <v>4270</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2441,7 +2441,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>5060</v>
+        <v>5240</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2449,10 +2449,10 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8626.5</v>
+        <v>8700</v>
       </c>
       <c r="G47" t="n">
-        <v>6279.5</v>
+        <v>6500</v>
       </c>
       <c r="H47" t="n">
         <v>12300</v>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -2529,7 +2529,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1902</v>
+        <v>1830</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>102.055</v>
+        <v>94.965</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>116.8</v>
+        <v>118.24</v>
       </c>
       <c r="G50" t="n">
         <v>79</v>
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1780</v>
+        <v>1755</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>14.73</v>
+        <v>15.425</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2705,7 +2705,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>5.2699</v>
+        <v>5.37</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1530</v>
+        <v>1610</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1.6973</v>
+        <v>1.6897</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>3.4044</v>
+        <v>3.25</v>
       </c>
       <c r="G55" t="n">
         <v>1.5</v>
@@ -2810,7 +2810,7 @@
         <v>6.5</v>
       </c>
       <c r="I55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>82.18000000000001</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>93.41556</v>
+        <v>93.66</v>
       </c>
       <c r="G56" t="n">
         <v>70</v>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>157.9</v>
+        <v>144.8807</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2897,16 +2897,16 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>95.66667</v>
+        <v>110.35294</v>
       </c>
       <c r="G57" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H57" t="n">
         <v>170</v>
       </c>
       <c r="I57" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>9.890700000000001</v>
+        <v>10.44</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1374</v>
+        <v>1478</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3025,7 +3025,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>9005</v>
+        <v>9210</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>5.39</v>
+        <v>4.655</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>222.26</v>
+        <v>231.04</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -3169,7 +3169,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>2960</v>
+        <v>3190</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -3209,7 +3209,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>181.39</v>
+        <v>183.325</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>4665</v>
+        <v>4680</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>358.195</v>
+        <v>364.19</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>526.3000500000001</v>
+        <v>525.97394</v>
       </c>
       <c r="G66" t="n">
         <v>215.88</v>
@@ -3333,7 +3333,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>70.03789999999999</v>
+        <v>69.01049999999999</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3369,7 +3369,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>346.9499</v>
+        <v>335.81</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>167.89</v>
+        <v>189.935</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3425,7 +3425,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>188.766</v>
+        <v>190.74129</v>
       </c>
       <c r="G69" t="n">
         <v>107.98</v>
@@ -3434,11 +3434,11 @@
         <v>480</v>
       </c>
       <c r="I69" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>23.895</v>
+        <v>24.865</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>110.97</v>
+        <v>105.22</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>120.08462</v>
+        <v>121.50538</v>
       </c>
       <c r="G71" t="n">
         <v>57</v>
@@ -3561,7 +3561,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>53.395</v>
+        <v>52.22</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3597,7 +3597,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>18.565</v>
+        <v>18.465</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -3633,7 +3633,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>121.18</v>
+        <v>111.84</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>23.375</v>
+        <v>21.515</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>3.19</v>
+        <v>3.35</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -3777,7 +3777,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>44.2</v>
+        <v>38.37</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -3825,7 +3825,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>118.075</v>
+        <v>115.03</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>43.2</v>
+        <v>42.37</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -3897,7 +3897,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>3.225</v>
+        <v>2.995</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -3945,7 +3945,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>6.7308</v>
+        <v>6.59</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -3993,7 +3993,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>39.73</v>
+        <v>40</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>341.8179</v>
+        <v>365.065</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>361.554</v>
+        <v>364.014</v>
       </c>
       <c r="G83" t="n">
         <v>201</v>
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>186.23</v>
+        <v>187.974</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -4097,7 +4097,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>181.3084</v>
+        <v>184.1884</v>
       </c>
       <c r="G84" t="n">
         <v>130</v>
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>87.33</v>
+        <v>83.47</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -4145,13 +4145,13 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>116.95385</v>
+        <v>116.25735</v>
       </c>
       <c r="G85" t="n">
-        <v>80.77634399999999</v>
+        <v>85.16468</v>
       </c>
       <c r="H85" t="n">
-        <v>171.78464</v>
+        <v>171.74367</v>
       </c>
       <c r="I85" t="n">
         <v>34</v>
@@ -4185,7 +4185,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>178.94</v>
+        <v>178.615</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -4221,7 +4221,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>138.5183</v>
+        <v>143.11</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -4229,16 +4229,16 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>216.33333</v>
+        <v>220.73685</v>
       </c>
       <c r="G87" t="n">
-        <v>75</v>
+        <v>117</v>
       </c>
       <c r="H87" t="n">
         <v>450</v>
       </c>
       <c r="I87" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>8.75</v>
+        <v>9.185</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -4277,13 +4277,13 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>11.689933</v>
+        <v>11.701622</v>
       </c>
       <c r="G88" t="n">
-        <v>7.7463994</v>
+        <v>7.7563353</v>
       </c>
       <c r="H88" t="n">
-        <v>14.045456</v>
+        <v>14.063471</v>
       </c>
       <c r="I88" t="n">
         <v>15</v>
@@ -4317,7 +4317,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>26.05</v>
+        <v>26.165</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -4353,7 +4353,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>44.64</v>
+        <v>44.27</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -4389,7 +4389,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>43.2</v>
+        <v>42.37</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>6.075</v>
+        <v>6.17</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -4485,7 +4485,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>6.92</v>
+        <v>6.78</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -4493,20 +4493,20 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>12.501751</v>
+        <v>12.429201</v>
       </c>
       <c r="G93" t="n">
-        <v>7.885828</v>
+        <v>7.8400655</v>
       </c>
       <c r="H93" t="n">
-        <v>18.205698</v>
+        <v>18.100048</v>
       </c>
       <c r="I93" t="n">
         <v>5</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -4533,7 +4533,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>21.315</v>
+        <v>17.865</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -4581,7 +4581,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>93.09</v>
+        <v>96.815</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -4629,7 +4629,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>4517.5</v>
+        <v>5175</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>41.435</v>
+        <v>43.5295</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -4717,7 +4717,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>163.36</v>
+        <v>161.465</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -4765,7 +4765,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>63.41</v>
+        <v>62.61</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>21.265</v>
+        <v>20.4</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -4861,7 +4861,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>143.25</v>
+        <v>139.11</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -4869,7 +4869,7 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>142.57143</v>
+        <v>144.04762</v>
       </c>
       <c r="G101" t="n">
         <v>119</v>
@@ -4909,7 +4909,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>10.19</v>
+        <v>10.21</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -4949,7 +4949,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>39.7397</v>
+        <v>38.315</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>50.66471</v>
+        <v>50.51765</v>
       </c>
       <c r="G103" t="n">
         <v>23</v>
@@ -4997,7 +4997,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>145.54</v>
+        <v>144.24</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -5018,7 +5018,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>105.02</v>
+        <v>105.52</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -5053,7 +5053,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>128.425</v>
+        <v>127.725</v>
       </c>
       <c r="G105" t="n">
         <v>81</v>
@@ -5093,7 +5093,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>7985</v>
+        <v>8255</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -5114,7 +5114,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -5141,7 +5141,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>16510</v>
+        <v>16140</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -5181,7 +5181,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>6.61</v>
+        <v>6.965</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -5189,7 +5189,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>6.723</v>
+        <v>6.623</v>
       </c>
       <c r="G108" t="n">
         <v>5</v>
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>119.475</v>
+        <v>116.17</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -5265,7 +5265,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>87.735</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -5313,7 +5313,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>20.6438</v>
+        <v>19.5</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>423.33</v>
+        <v>414</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -5369,13 +5369,13 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>465.07217</v>
+        <v>462.37326</v>
       </c>
       <c r="G112" t="n">
-        <v>403.03296</v>
+        <v>400.6941</v>
       </c>
       <c r="H112" t="n">
-        <v>537.0068</v>
+        <v>533.89044</v>
       </c>
       <c r="I112" t="n">
         <v>14</v>
@@ -5409,7 +5409,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>84.88</v>
+        <v>80.69</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -5457,7 +5457,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>240.62</v>
+        <v>203.52</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -5465,7 +5465,7 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>266.35535</v>
+        <v>279.62363</v>
       </c>
       <c r="G114" t="n">
         <v>126</v>
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>22.805</v>
+        <v>19.425</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -5553,7 +5553,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>17.685</v>
+        <v>17.24</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -5589,7 +5589,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>88.67</v>
+        <v>81.55</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>82.12</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -5645,7 +5645,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>97.97499999999999</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="G118" t="n">
         <v>75</v>
@@ -5685,7 +5685,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>158.485</v>
+        <v>157.01</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -5706,7 +5706,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>hold</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -5733,7 +5733,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>15.075</v>
+        <v>15.14</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -5741,7 +5741,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>16.736</v>
+        <v>16.632</v>
       </c>
       <c r="G120" t="n">
         <v>12</v>
@@ -5781,7 +5781,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>45.39</v>
+        <v>44.22</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -5817,7 +5817,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>73.63</v>
+        <v>72.575</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -5853,7 +5853,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>32.485</v>
+        <v>32.6499</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -5889,7 +5889,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>24.215</v>
+        <v>23.85</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>33.215</v>
+        <v>29.855</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -5985,7 +5985,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>25.705</v>
+        <v>26.23</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -6033,7 +6033,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>175.37</v>
+        <v>171.955</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -6069,7 +6069,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>76.715</v>
+        <v>79.345</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -6077,13 +6077,13 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>115.641335</v>
+        <v>113.88258</v>
       </c>
       <c r="G128" t="n">
-        <v>83.94277</v>
+        <v>83.85955</v>
       </c>
       <c r="H128" t="n">
-        <v>148.62057</v>
+        <v>150.0595</v>
       </c>
       <c r="I128" t="n">
         <v>9</v>
@@ -6117,7 +6117,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>138.595</v>
+        <v>138.25</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -6153,7 +6153,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>70.06999999999999</v>
+        <v>63.8</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -6201,7 +6201,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>83.98999999999999</v>
+        <v>82.913</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -6249,7 +6249,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>86.68000000000001</v>
+        <v>83.895</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -6285,7 +6285,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>62.7</v>
+        <v>61.565</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>82.7431</v>
+        <v>77.5</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -6341,7 +6341,7 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>105.02083</v>
+        <v>105.1875</v>
       </c>
       <c r="G134" t="n">
         <v>50</v>
@@ -6381,7 +6381,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>86.31999999999999</v>
+        <v>85.785</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>81.625</v>
+        <v>82.005</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -6453,7 +6453,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>1742.9</v>
+        <v>1660</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -6461,16 +6461,16 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>2195.1438</v>
+        <v>2146.371</v>
       </c>
       <c r="G137" t="n">
-        <v>903.1520400000001</v>
+        <v>897.9109</v>
       </c>
       <c r="H137" t="n">
-        <v>2899.051</v>
+        <v>2882.2273</v>
       </c>
       <c r="I137" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J137" t="inlineStr">
         <is>
@@ -6501,7 +6501,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>108.5173</v>
+        <v>107.1</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>95.355</v>
+        <v>95.68000000000001</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>42.26</v>
+        <v>35.405</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -6581,10 +6581,10 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>80.1875</v>
+        <v>78.3125</v>
       </c>
       <c r="G140" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H140" t="n">
         <v>131</v>
@@ -6621,7 +6621,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>14330</v>
+        <v>15380</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -6661,7 +6661,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>216.45</v>
+        <v>209.47</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>11.299</v>
+        <v>10.25</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -6705,13 +6705,13 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>19.436132</v>
+        <v>19.360693</v>
       </c>
       <c r="G143" t="n">
-        <v>19.436132</v>
+        <v>19.360693</v>
       </c>
       <c r="H143" t="n">
-        <v>19.436132</v>
+        <v>19.360693</v>
       </c>
       <c r="I143" t="n">
         <v>1</v>
@@ -6745,7 +6745,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>237.34</v>
+        <v>236.22</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -6781,7 +6781,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>13.7282</v>
+        <v>13.275</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -6789,7 +6789,7 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>18.58696</v>
+        <v>18.5</v>
       </c>
       <c r="G145" t="n">
         <v>10</v>
@@ -6829,7 +6829,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>552.4</v>
+        <v>543.115</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -6837,13 +6837,13 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>614.85425</v>
+        <v>613.05566</v>
       </c>
       <c r="G146" t="n">
-        <v>425.73666</v>
+        <v>423.26602</v>
       </c>
       <c r="H146" t="n">
-        <v>729.8343</v>
+        <v>725.59894</v>
       </c>
       <c r="I146" t="n">
         <v>39</v>
@@ -6877,7 +6877,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>242.06</v>
+        <v>231.92</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -6885,7 +6885,7 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>285.72308</v>
+        <v>286.44104</v>
       </c>
       <c r="G147" t="n">
         <v>125</v>
@@ -6925,7 +6925,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>160.84</v>
+        <v>159.84</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -6961,7 +6961,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>178.36</v>
+        <v>173.98</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>189.6699</v>
+        <v>190.45</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -7045,7 +7045,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>244.13</v>
+        <v>241.63</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>425.42</v>
+        <v>399.4102</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -7117,7 +7117,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>62.16</v>
+        <v>52.505</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -7125,7 +7125,7 @@
         </is>
       </c>
       <c r="F153" t="n">
-        <v>59.76939</v>
+        <v>59.8103</v>
       </c>
       <c r="G153" t="n">
         <v>36</v>
@@ -7165,7 +7165,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>28.38</v>
+        <v>28.742</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -7213,7 +7213,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>138.8614</v>
+        <v>136.11</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -7221,13 +7221,13 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>217.84212</v>
+        <v>217.42105</v>
       </c>
       <c r="G155" t="n">
         <v>106</v>
       </c>
       <c r="H155" t="n">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="I155" t="n">
         <v>19</v>
@@ -7261,7 +7261,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>14.795</v>
+        <v>14.655</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -7309,7 +7309,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>276.8608</v>
+        <v>275.575</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -7357,7 +7357,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>62.076</v>
+        <v>58.4</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -7393,7 +7393,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>43.175</v>
+        <v>43.915</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -7441,7 +7441,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>272.27</v>
+        <v>290.44</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -7449,7 +7449,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>270.60587</v>
+        <v>272.22354</v>
       </c>
       <c r="G160" t="n">
         <v>190</v>
@@ -7489,7 +7489,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>181.5051</v>
+        <v>183.07</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>95.7</v>
+        <v>91.23</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -7573,7 +7573,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>16.4563</v>
+        <v>18.355</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -7594,7 +7594,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -7621,7 +7621,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>78.5883</v>
+        <v>77.16</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -7657,7 +7657,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>188.065</v>
+        <v>181.209</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -7665,7 +7665,7 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>196.55414</v>
+        <v>197.58862</v>
       </c>
       <c r="G165" t="n">
         <v>95</v>
@@ -7709,7 +7709,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>112.9395</v>
+        <v>110.99</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -7745,7 +7745,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>35.495</v>
+        <v>35.555</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -7781,7 +7781,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>34.855</v>
+        <v>35.36</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -7817,7 +7817,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>553.8</v>
+        <v>542.6</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -7853,7 +7853,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>315.0301</v>
+        <v>323.4</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -7861,7 +7861,7 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>321.35</v>
+        <v>327.85</v>
       </c>
       <c r="G170" t="n">
         <v>110</v>
@@ -7901,7 +7901,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>106.085</v>
+        <v>106.635</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -7949,7 +7949,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>53.765</v>
+        <v>50.75</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -7997,7 +7997,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>309.69</v>
+        <v>321.83</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -8045,7 +8045,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>2.9</v>
+        <v>2.935</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -8097,7 +8097,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>126.85</v>
+        <v>129.315</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -8105,13 +8105,13 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>229.07143</v>
+        <v>225.14285</v>
       </c>
       <c r="G175" t="n">
         <v>125</v>
       </c>
       <c r="H175" t="n">
-        <v>450</v>
+        <v>435</v>
       </c>
       <c r="I175" t="n">
         <v>14</v>
@@ -8145,7 +8145,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>30.675</v>
+        <v>30.25</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -8153,13 +8153,13 @@
         </is>
       </c>
       <c r="F176" t="n">
-        <v>35.6875</v>
+        <v>34.6875</v>
       </c>
       <c r="G176" t="n">
         <v>29</v>
       </c>
       <c r="H176" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="I176" t="n">
         <v>16</v>
@@ -8193,7 +8193,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>18.74</v>
+        <v>18.32</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -8229,7 +8229,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>32.3499</v>
+        <v>29.205</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -8277,7 +8277,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>85.8908</v>
+        <v>84.73</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -8313,7 +8313,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>565.5650000000001</v>
+        <v>566.3049999999999</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -8321,7 +8321,7 @@
         </is>
       </c>
       <c r="F180" t="n">
-        <v>754.14246</v>
+        <v>754.77405</v>
       </c>
       <c r="G180" t="n">
         <v>580</v>
@@ -8361,7 +8361,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>221.53</v>
+        <v>218.42</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -8397,7 +8397,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>764.9450000000001</v>
+        <v>762.3209000000001</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -8433,7 +8433,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>186.01</v>
+        <v>178.515</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -8481,7 +8481,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>92.52</v>
+        <v>95.62</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -8489,13 +8489,13 @@
         </is>
       </c>
       <c r="F184" t="n">
-        <v>150.57062</v>
+        <v>148.82843</v>
       </c>
       <c r="G184" t="n">
-        <v>80.27906</v>
+        <v>80.25991</v>
       </c>
       <c r="H184" t="n">
-        <v>206.68387</v>
+        <v>206.63457</v>
       </c>
       <c r="I184" t="n">
         <v>32</v>
@@ -8529,7 +8529,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>29.16</v>
+        <v>28.045</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -8537,13 +8537,13 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>39.74984</v>
+        <v>39.717564</v>
       </c>
       <c r="G185" t="n">
-        <v>25.13461</v>
+        <v>25.128614</v>
       </c>
       <c r="H185" t="n">
-        <v>54.780876</v>
+        <v>54.76781</v>
       </c>
       <c r="I185" t="n">
         <v>35</v>
@@ -8577,7 +8577,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>14820</v>
+        <v>14320</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -8617,7 +8617,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>142.36</v>
+        <v>140.62</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>7.565</v>
+        <v>7.8</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -8713,7 +8713,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>10.1105</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -8734,7 +8734,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -8761,7 +8761,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>220.225</v>
+        <v>197.105</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -8809,7 +8809,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>62.27</v>
+        <v>62.355</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -8830,7 +8830,7 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -8857,7 +8857,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>106.145</v>
+        <v>102.76</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -8905,7 +8905,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>67.40000000000001</v>
+        <v>62.365</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -8913,7 +8913,7 @@
         </is>
       </c>
       <c r="F193" t="n">
-        <v>112.94118</v>
+        <v>112.64706</v>
       </c>
       <c r="G193" t="n">
         <v>64</v>
@@ -8953,7 +8953,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>92.37</v>
+        <v>97.43000000000001</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -8989,7 +8989,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>66.98999999999999</v>
+        <v>67.27</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -9025,7 +9025,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>9.630000000000001</v>
+        <v>10.91</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -9046,7 +9046,7 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -9073,7 +9073,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>192.832</v>
+        <v>189.905</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -9121,7 +9121,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>48.27</v>
+        <v>44.31</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -9157,7 +9157,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>190.515</v>
+        <v>182.13</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -9205,7 +9205,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>179.6</v>
+        <v>170.68</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -9253,7 +9253,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>58.925</v>
+        <v>60.719</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -9261,7 +9261,7 @@
         </is>
       </c>
       <c r="F201" t="n">
-        <v>66.56522</v>
+        <v>66.82608999999999</v>
       </c>
       <c r="G201" t="n">
         <v>55</v>
@@ -9301,7 +9301,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>5.715</v>
+        <v>5.365</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -9349,7 +9349,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>84.22499999999999</v>
+        <v>87.12</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -9397,7 +9397,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>211.07</v>
+        <v>206.43</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -9405,7 +9405,7 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>274.04</v>
+        <v>274.84616</v>
       </c>
       <c r="G204" t="n">
         <v>246</v>
@@ -9414,7 +9414,7 @@
         <v>305</v>
       </c>
       <c r="I204" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J204" t="inlineStr">
         <is>
@@ -9445,7 +9445,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>200.905</v>
+        <v>209.66</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -9453,7 +9453,7 @@
         </is>
       </c>
       <c r="F205" t="n">
-        <v>218.08333</v>
+        <v>218.29167</v>
       </c>
       <c r="G205" t="n">
         <v>175</v>
@@ -9493,7 +9493,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>86.605</v>
+        <v>86.14</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -9541,7 +9541,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>397.6578</v>
+        <v>396.995</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -9589,7 +9589,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>17410</v>
+        <v>18180</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -9629,7 +9629,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>628.715</v>
+        <v>669.42</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -9637,7 +9637,7 @@
         </is>
       </c>
       <c r="F209" t="n">
-        <v>665.3477</v>
+        <v>666.71136</v>
       </c>
       <c r="G209" t="n">
         <v>500</v>
@@ -9677,7 +9677,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>118.59</v>
+        <v>113.285</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -9685,13 +9685,13 @@
         </is>
       </c>
       <c r="F210" t="n">
-        <v>188.47086</v>
+        <v>187.12779</v>
       </c>
       <c r="G210" t="n">
-        <v>92.91471</v>
+        <v>95.19119999999999</v>
       </c>
       <c r="H210" t="n">
-        <v>240.65308</v>
+        <v>238.1918</v>
       </c>
       <c r="I210" t="n">
         <v>39</v>
@@ -9725,7 +9725,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>476.89</v>
+        <v>457.8686</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -9733,7 +9733,7 @@
         </is>
       </c>
       <c r="F211" t="n">
-        <v>613.0916999999999</v>
+        <v>613.8449000000001</v>
       </c>
       <c r="G211" t="n">
         <v>365</v>
@@ -9742,7 +9742,7 @@
         <v>1250</v>
       </c>
       <c r="I211" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J211" t="inlineStr">
         <is>
@@ -9773,7 +9773,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>83.325</v>
+        <v>82.01000000000001</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -9821,7 +9821,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>13.9828</v>
+        <v>13.9464</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -9869,7 +9869,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>206.43</v>
+        <v>200.35</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -9877,7 +9877,7 @@
         </is>
       </c>
       <c r="F214" t="n">
-        <v>273.538</v>
+        <v>275.30466</v>
       </c>
       <c r="G214" t="n">
         <v>150</v>
@@ -9917,7 +9917,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>48.71</v>
+        <v>43.94</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -9965,7 +9965,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>160.63</v>
+        <v>163.1403</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -9986,7 +9986,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -10013,7 +10013,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>1486.77</v>
+        <v>1543.01</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
         </is>
       </c>
       <c r="F217" t="n">
-        <v>2126.1738</v>
+        <v>2125.087</v>
       </c>
       <c r="G217" t="n">
         <v>1000</v>
@@ -10061,7 +10061,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>272.92</v>
+        <v>269.01</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -10109,7 +10109,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>67.84</v>
+        <v>73.95</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -10117,20 +10117,20 @@
         </is>
       </c>
       <c r="F219" t="n">
-        <v>98.80342</v>
+        <v>98.681175</v>
       </c>
       <c r="G219" t="n">
-        <v>82.12031</v>
+        <v>82.13291</v>
       </c>
       <c r="H219" t="n">
-        <v>123.465096</v>
+        <v>123.48404</v>
       </c>
       <c r="I219" t="n">
         <v>12</v>
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -10157,7 +10157,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>110.97</v>
+        <v>109.52</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -10165,16 +10165,16 @@
         </is>
       </c>
       <c r="F220" t="n">
-        <v>136.27274</v>
+        <v>137.73914</v>
       </c>
       <c r="G220" t="n">
         <v>115</v>
       </c>
       <c r="H220" t="n">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="I220" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J220" t="inlineStr">
         <is>
@@ -10205,7 +10205,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>114.74</v>
+        <v>106.665</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -10213,7 +10213,7 @@
         </is>
       </c>
       <c r="F221" t="n">
-        <v>161.28261</v>
+        <v>161.41304</v>
       </c>
       <c r="G221" t="n">
         <v>95</v>
@@ -10253,7 +10253,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>11.55</v>
+        <v>10.85</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -10293,7 +10293,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>222.19</v>
+        <v>197.245</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -10341,7 +10341,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>135.845</v>
+        <v>132.875</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -10362,7 +10362,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -10389,7 +10389,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>53.29</v>
+        <v>59.45</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -10437,7 +10437,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>444.5</v>
+        <v>434.555</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -10485,7 +10485,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>184.62</v>
+        <v>219.918</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -10493,16 +10493,16 @@
         </is>
       </c>
       <c r="F227" t="n">
-        <v>210.535</v>
+        <v>229.30612</v>
       </c>
       <c r="G227" t="n">
-        <v>103.25</v>
+        <v>119</v>
       </c>
       <c r="H227" t="n">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="I227" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J227" t="inlineStr">
         <is>
@@ -10533,7 +10533,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>145.258</v>
+        <v>147.66</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -10581,7 +10581,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>269.065</v>
+        <v>262.16</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -10589,7 +10589,7 @@
         </is>
       </c>
       <c r="F229" t="n">
-        <v>316.0645</v>
+        <v>315.3871</v>
       </c>
       <c r="G229" t="n">
         <v>250</v>
@@ -10629,7 +10629,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>8.065</v>
+        <v>7.96</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -10677,7 +10677,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>50.145</v>
+        <v>50.615</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -10729,7 +10729,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>104.845</v>
+        <v>96.53</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -10765,7 +10765,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>1.015</v>
+        <v>1.0691</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -10773,7 +10773,7 @@
         </is>
       </c>
       <c r="F233" t="n">
-        <v>1.20333</v>
+        <v>1.2</v>
       </c>
       <c r="G233" t="n">
         <v>0.9</v>
@@ -10782,11 +10782,11 @@
         <v>1.5</v>
       </c>
       <c r="I233" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>underperform</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -10813,7 +10813,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>285.45</v>
+        <v>282.06</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -10849,7 +10849,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>221.865</v>
+        <v>217.995</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -10857,7 +10857,7 @@
         </is>
       </c>
       <c r="F235" t="n">
-        <v>235.57484</v>
+        <v>236.22</v>
       </c>
       <c r="G235" t="n">
         <v>165</v>
@@ -10897,7 +10897,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>91.61499999999999</v>
+        <v>89.12</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -10945,7 +10945,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>206.15</v>
+        <v>257.89</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -10953,7 +10953,7 @@
         </is>
       </c>
       <c r="F237" t="n">
-        <v>243.98425</v>
+        <v>266.48364</v>
       </c>
       <c r="G237" t="n">
         <v>160</v>
@@ -10962,7 +10962,7 @@
         <v>475</v>
       </c>
       <c r="I237" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J237" t="inlineStr">
         <is>
@@ -10993,7 +10993,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>34.055</v>
+        <v>37.135</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -11001,7 +11001,7 @@
         </is>
       </c>
       <c r="F238" t="n">
-        <v>43.2</v>
+        <v>43.12</v>
       </c>
       <c r="G238" t="n">
         <v>29</v>
@@ -11041,7 +11041,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>17.725</v>
+        <v>19.925</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -11049,7 +11049,7 @@
         </is>
       </c>
       <c r="F239" t="n">
-        <v>22.02743</v>
+        <v>22.0275</v>
       </c>
       <c r="G239" t="n">
         <v>17.4</v>
@@ -11089,7 +11089,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>161.75</v>
+        <v>163.835</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -11137,7 +11137,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>335.93</v>
+        <v>322.68</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -11185,7 +11185,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>16.9138</v>
+        <v>14.925</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -11233,7 +11233,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>4.315</v>
+        <v>4.665</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -11241,13 +11241,13 @@
         </is>
       </c>
       <c r="F243" t="n">
-        <v>5.4561934</v>
+        <v>5.5665975</v>
       </c>
       <c r="G243" t="n">
-        <v>5.0050464</v>
+        <v>5.0090327</v>
       </c>
       <c r="H243" t="n">
-        <v>5.9500794</v>
+        <v>6.095453</v>
       </c>
       <c r="I243" t="n">
         <v>5</v>
@@ -11281,7 +11281,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>415.035</v>
+        <v>415.34</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -11302,7 +11302,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -11329,7 +11329,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>67.92</v>
+        <v>69.861</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -11377,7 +11377,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>192.84</v>
+        <v>199.205</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -11425,7 +11425,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>808.76</v>
+        <v>780.015</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -11433,7 +11433,7 @@
         </is>
       </c>
       <c r="F247" t="n">
-        <v>979.2196</v>
+        <v>975.60614</v>
       </c>
       <c r="G247" t="n">
         <v>575</v>
@@ -11473,7 +11473,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>3.005</v>
+        <v>2.89</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -11521,7 +11521,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>35.405</v>
+        <v>36.735</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -11557,7 +11557,7 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>1994.49</v>
+        <v>1944.04</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -11605,7 +11605,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>14.725</v>
+        <v>14.75</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -11653,7 +11653,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>1248.91</v>
+        <v>1169.405</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -11701,7 +11701,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>23.615</v>
+        <v>22.14</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -11749,7 +11749,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>79.045</v>
+        <v>74.145</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -11757,13 +11757,13 @@
         </is>
       </c>
       <c r="F254" t="n">
-        <v>71.72727</v>
+        <v>72.04545</v>
       </c>
       <c r="G254" t="n">
         <v>30</v>
       </c>
       <c r="H254" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I254" t="n">
         <v>22</v>
@@ -11797,7 +11797,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>352.81</v>
+        <v>358.67</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -11845,7 +11845,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>489.875</v>
+        <v>503.33</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -11893,7 +11893,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>231.69</v>
+        <v>231.05</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -11941,7 +11941,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>67.642</v>
+        <v>67.2</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -11989,7 +11989,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>1715</v>
+        <v>1790</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -12029,7 +12029,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>266.04</v>
+        <v>260.47</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -12077,7 +12077,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>598.395</v>
+        <v>588.765</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -12085,13 +12085,13 @@
         </is>
       </c>
       <c r="F261" t="n">
-        <v>667.2973</v>
+        <v>670.91895</v>
       </c>
       <c r="G261" t="n">
         <v>550</v>
       </c>
       <c r="H261" t="n">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="I261" t="n">
         <v>37</v>
@@ -12125,7 +12125,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>65.19499999999999</v>
+        <v>65.41</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -12133,13 +12133,13 @@
         </is>
       </c>
       <c r="F262" t="n">
-        <v>74.53071</v>
+        <v>74.09819</v>
       </c>
       <c r="G262" t="n">
-        <v>70.58955</v>
+        <v>70.1799</v>
       </c>
       <c r="H262" t="n">
-        <v>77.86365000000001</v>
+        <v>77.41179</v>
       </c>
       <c r="I262" t="n">
         <v>4</v>
@@ -12173,7 +12173,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>337.46</v>
+        <v>328.29</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -12269,7 +12269,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>154.82</v>
+        <v>150.03</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -12277,7 +12277,7 @@
         </is>
       </c>
       <c r="F265" t="n">
-        <v>147.76923</v>
+        <v>148.73077</v>
       </c>
       <c r="G265" t="n">
         <v>105</v>
@@ -12317,7 +12317,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>209.69</v>
+        <v>209.6</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -12365,7 +12365,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>330.126</v>
+        <v>326.78</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -12413,7 +12413,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>534.33</v>
+        <v>529.58</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -12449,7 +12449,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>959.91</v>
+        <v>945.8099999999999</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -12470,7 +12470,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -12497,7 +12497,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>58.19</v>
+        <v>57.61</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>94.755</v>
+        <v>90.97</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -12541,13 +12541,13 @@
         </is>
       </c>
       <c r="F271" t="n">
-        <v>106.42857</v>
+        <v>106.28571</v>
       </c>
       <c r="G271" t="n">
         <v>76</v>
       </c>
       <c r="H271" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I271" t="n">
         <v>7</v>
@@ -12581,7 +12581,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>382.385</v>
+        <v>378.855</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -12589,16 +12589,16 @@
         </is>
       </c>
       <c r="F272" t="n">
-        <v>418.22223</v>
+        <v>419.36163</v>
       </c>
       <c r="G272" t="n">
         <v>330</v>
       </c>
       <c r="H272" t="n">
-        <v>450</v>
+        <v>466</v>
       </c>
       <c r="I272" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J272" t="inlineStr">
         <is>
@@ -12629,7 +12629,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>110.355</v>
+        <v>108.13</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -12677,7 +12677,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>298.605</v>
+        <v>291.74</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -12713,7 +12713,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>36780</v>
+        <v>36640</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -12753,7 +12753,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>21900</v>
+        <v>21450</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -12793,7 +12793,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>627.4299999999999</v>
+        <v>612.5</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -12841,7 +12841,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>35580</v>
+        <v>37200</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -12881,7 +12881,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>355.685</v>
+        <v>356.67</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -12902,7 +12902,7 @@
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -12929,7 +12929,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>709.53</v>
+        <v>707.6903</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -12965,7 +12965,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>62.555</v>
+        <v>64.59</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -13001,7 +13001,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>132.96</v>
+        <v>132.71</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -13022,7 +13022,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -13049,7 +13049,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>29.3</v>
+        <v>30.2275</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -13057,13 +13057,13 @@
         </is>
       </c>
       <c r="F283" t="n">
-        <v>23.4125</v>
+        <v>29.45625</v>
       </c>
       <c r="G283" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H283" t="n">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="I283" t="n">
         <v>16</v>
@@ -13097,7 +13097,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>558.37</v>
+        <v>557.65</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -13145,7 +13145,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>485.485</v>
+        <v>490.035</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -13153,7 +13153,7 @@
         </is>
       </c>
       <c r="F285" t="n">
-        <v>522.7273</v>
+        <v>526.8182</v>
       </c>
       <c r="G285" t="n">
         <v>476</v>
@@ -13193,7 +13193,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>105.7</v>
+        <v>104.88</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -13241,7 +13241,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>115.49</v>
+        <v>110.58</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -13289,7 +13289,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>3.505</v>
+        <v>3.065</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -13310,7 +13310,7 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">
@@ -13337,7 +13337,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>925.1799999999999</v>
+        <v>942</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -13345,7 +13345,7 @@
         </is>
       </c>
       <c r="F289" t="n">
-        <v>1515.1136</v>
+        <v>1513.409</v>
       </c>
       <c r="G289" t="n">
         <v>361</v>
@@ -13385,7 +13385,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>14.585</v>
+        <v>14.595</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -13393,10 +13393,10 @@
         </is>
       </c>
       <c r="F290" t="n">
-        <v>13.56</v>
+        <v>14.79333</v>
       </c>
       <c r="G290" t="n">
-        <v>9.300000000000001</v>
+        <v>13</v>
       </c>
       <c r="H290" t="n">
         <v>15.78</v>
@@ -13433,7 +13433,7 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>83.605</v>
+        <v>75.8535</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -13481,7 +13481,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>91.5</v>
+        <v>90.965</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -13529,7 +13529,7 @@
         </is>
       </c>
       <c r="D293" t="n">
-        <v>38.46</v>
+        <v>40.05</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="D294" t="n">
-        <v>147.68</v>
+        <v>147.8</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -13625,7 +13625,7 @@
         </is>
       </c>
       <c r="D295" t="n">
-        <v>292.365</v>
+        <v>291.25</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -13646,7 +13646,7 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="K295" t="inlineStr">
@@ -13673,7 +13673,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>169.1597</v>
+        <v>162.65</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -13721,7 +13721,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>97.91</v>
+        <v>93.59</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -13769,7 +13769,7 @@
         </is>
       </c>
       <c r="D298" t="n">
-        <v>216.045</v>
+        <v>215.82</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -13777,7 +13777,7 @@
         </is>
       </c>
       <c r="F298" t="n">
-        <v>245.33333</v>
+        <v>247.25</v>
       </c>
       <c r="G298" t="n">
         <v>177</v>
@@ -13817,7 +13817,7 @@
         </is>
       </c>
       <c r="D299" t="n">
-        <v>129.52</v>
+        <v>123.325</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -13838,7 +13838,7 @@
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -13865,7 +13865,7 @@
         </is>
       </c>
       <c r="D300" t="n">
-        <v>92.48999999999999</v>
+        <v>92.89</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -13913,7 +13913,7 @@
         </is>
       </c>
       <c r="D301" t="n">
-        <v>477.38</v>
+        <v>442.98</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -13921,7 +13921,7 @@
         </is>
       </c>
       <c r="F301" t="n">
-        <v>641.02856</v>
+        <v>640.3143</v>
       </c>
       <c r="G301" t="n">
         <v>358</v>
@@ -13961,7 +13961,7 @@
         </is>
       </c>
       <c r="D302" t="n">
-        <v>259.25</v>
+        <v>252.74</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -13969,7 +13969,7 @@
         </is>
       </c>
       <c r="F302" t="n">
-        <v>323.67743</v>
+        <v>324.7097</v>
       </c>
       <c r="G302" t="n">
         <v>225</v>
@@ -14009,7 +14009,7 @@
         </is>
       </c>
       <c r="D303" t="n">
-        <v>40.69</v>
+        <v>39.47</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -14045,7 +14045,7 @@
         </is>
       </c>
       <c r="D304" t="n">
-        <v>79.72499999999999</v>
+        <v>75.01000000000001</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -14053,7 +14053,7 @@
         </is>
       </c>
       <c r="F304" t="n">
-        <v>101.78391</v>
+        <v>101.84913</v>
       </c>
       <c r="G304" t="n">
         <v>70</v>
@@ -14093,7 +14093,7 @@
         </is>
       </c>
       <c r="D305" t="n">
-        <v>133.52</v>
+        <v>124.5</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -14141,7 +14141,7 @@
         </is>
       </c>
       <c r="D306" t="n">
-        <v>393.32</v>
+        <v>383.8101</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -14162,7 +14162,7 @@
       </c>
       <c r="J306" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>hold</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
@@ -14189,7 +14189,7 @@
         </is>
       </c>
       <c r="D307" t="n">
-        <v>9.654999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -14197,13 +14197,13 @@
         </is>
       </c>
       <c r="F307" t="n">
-        <v>12.094268</v>
+        <v>12.049841</v>
       </c>
       <c r="G307" t="n">
-        <v>9.483121000000001</v>
+        <v>9.448286</v>
       </c>
       <c r="H307" t="n">
-        <v>14.265886</v>
+        <v>14.213483</v>
       </c>
       <c r="I307" t="n">
         <v>3</v>
@@ -14237,7 +14237,7 @@
         </is>
       </c>
       <c r="D308" t="n">
-        <v>217.08</v>
+        <v>206.57</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -14245,13 +14245,13 @@
         </is>
       </c>
       <c r="F308" t="n">
-        <v>166.76906</v>
+        <v>169.05853</v>
       </c>
       <c r="G308" t="n">
         <v>126.97628</v>
       </c>
       <c r="H308" t="n">
-        <v>247.03557</v>
+        <v>275</v>
       </c>
       <c r="I308" t="n">
         <v>17</v>
@@ -14285,7 +14285,7 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>144.31</v>
+        <v>143.83</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -14293,7 +14293,7 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>246.42635</v>
+        <v>244.11761</v>
       </c>
       <c r="G309" t="n">
         <v>110</v>
@@ -14302,7 +14302,7 @@
         <v>400</v>
       </c>
       <c r="I309" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J309" t="inlineStr">
         <is>
@@ -14333,7 +14333,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>173.21</v>
+        <v>184.0701</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -14381,7 +14381,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>69.53</v>
+        <v>65.75</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -14421,7 +14421,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>288.83</v>
+        <v>283.14</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -14442,7 +14442,7 @@
       </c>
       <c r="J312" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K312" t="inlineStr">
@@ -14469,7 +14469,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>50.23</v>
+        <v>42.06</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -14517,7 +14517,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>1055.21</v>
+        <v>1015.2</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -14565,7 +14565,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>78.95999999999999</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -14573,7 +14573,7 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>120.77273</v>
+        <v>121.09091</v>
       </c>
       <c r="G315" t="n">
         <v>100</v>
@@ -14613,7 +14613,7 @@
         </is>
       </c>
       <c r="D316" t="n">
-        <v>102.92</v>
+        <v>102.83</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -14649,7 +14649,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>110.335</v>
+        <v>110.055</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -14685,7 +14685,7 @@
         </is>
       </c>
       <c r="D318" t="n">
-        <v>343.25</v>
+        <v>332.77</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -14733,7 +14733,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>262.975</v>
+        <v>253.88</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -14781,7 +14781,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>404.59</v>
+        <v>424.89</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -14789,13 +14789,13 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>560.1738</v>
+        <v>544.9723</v>
       </c>
       <c r="G320" t="n">
         <v>414.77</v>
       </c>
       <c r="H320" t="n">
-        <v>650</v>
+        <v>633</v>
       </c>
       <c r="I320" t="n">
         <v>26</v>

</xml_diff>